<commit_message>
Chat Completions support added
</commit_message>
<xml_diff>
--- a/examples/default_imports/cyberprompt_ai_default_endpoints.xlsx
+++ b/examples/default_imports/cyberprompt_ai_default_endpoints.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,30 +451,35 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>request_mode</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>headers</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>body</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>response_paths</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>response_type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>additional_variables</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>api_token</t>
         </is>
@@ -503,126 +508,247 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>responses</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>{"Content-Type": "application/json", "Authorization": "Bearer {{API_TOKEN}}"}</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>{"model": "{{MODEL_NAME}}", "input": "{{PROMPT}}", "max_output_tokens": 1000, "temperature": 0.7}</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>$output[1].content[0].text</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anthropic Messages - Sonnet</t>
+          <t>OpenAI Chat Completion - GPT 4.1 Mini</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://api.anthropic.com/v1/messages</t>
+          <t>https://api.openai.com/v1/chat/completions</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>claude-sonnet-4-5</t>
+          <t>gpt-4.1-mini</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{"Content-Type": "application/json", "x-api-key": "{{API_TOKEN}}", "anthropic-version": "2023-06-01"}</t>
+          <t>completions</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>{"Content-Type": "application/json", "Authorization": "Bearer {{API_TOKEN}}"}</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>{"model": "{{MODEL_NAME}}", "messages": [{"role": "user", "content": "{{PROMPT}}"}], "max_tokens": 1000, "temperature": 0.7}</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>$content[0].text</t>
-        </is>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>$choices[0].message.content</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>json</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Anthropic Messages - Sonnet</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://api.anthropic.com/v1/messages</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4-5</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>responses</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json", "x-api-key": "{{API_TOKEN}}", "anthropic-version": "2023-06-01"}</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>{"model": "{{MODEL_NAME}}", "messages": [{"role": "user", "content": "{{PROMPT}}"}], "max_tokens": 1000, "temperature": 0.7}</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>$content[0].text</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Gemini Generate Content - Flash</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Google Gemini</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>https://generativelanguage.googleapis.com/v1beta/models/gemini-2.0-flash:generateContent?key={{API_TOKEN}}</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>gemini-2.0-flash</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>responses</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>{"Content-Type": "application/json"}</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>{"contents": [{"parts": [{"text": "{{PROMPT}}"}]}]}</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>$candidates[0].content.parts[0].text</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Azure OpenAI Chat Completion - Example</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Azure Foundry</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://YOUR_RESOURCE.openai.azure.com/openai/deployments/{{MODEL_NAME}}/chat/completions?api-version=2024-06-01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>gpt-4.1-mini</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>completions</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json", "api-key": "{{API_TOKEN}}"}</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>{"messages": [{"role": "system", "content": "You are a helpful assistant."}, {"role": "user", "content": "{{PROMPT}}"}], "max_tokens": 1000, "temperature": 0.7}</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>$choices[0].message.content</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>